<commit_message>
Update comic_list.xlsx via Book Manager
</commit_message>
<xml_diff>
--- a/comic_list.xlsx
+++ b/comic_list.xlsx
@@ -4,7 +4,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Đội quân nhí nhố" sheetId="1" r:id="rId1"/>
-    <sheet name="_meta" sheetId="2" r:id="rId2" state="hidden"/>
+    <sheet name="Yugioh" sheetId="2" r:id="rId2"/>
+    <sheet name="Thần đồng đất Việt" sheetId="3" r:id="rId3"/>
+    <sheet name="Conan" sheetId="4" r:id="rId4"/>
+    <sheet name="_meta" sheetId="5" r:id="rId5" state="hidden"/>
   </sheets>
 </workbook>
 </file>
@@ -854,7 +857,88 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C1"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Item</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C1"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Item</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C1"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Item</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -878,9 +962,42 @@
         <v>Đẹp|Cũ|Chưa có|Đẹp, thừa cũ</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Yugioh</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Thần đồng đất Việt</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Conan</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>